<commit_message>
SPM-43: review requests only once the event is approved
Since SPM-54 a venue can only be requested after the event is approved.
Booking Requests now leaves out a pending request whose event is still
Submitted or Under review, and the server refuses to approve one.

- prisma/seed.ts: drop the two base-seed pending requests on events not yet
  approved (Straits Medical Journal Club, Nusantara Developer Summit).
  scripts/remove-pre-approval-bookings.ts removes them from a database
  seeded earlier, without a reseed.
- SPM-43 fixtures: SPM43 Two-Day Forum starts as Planning; new events
  SPM43 Policy Briefing (TC15) and SPM43 Alumni Lecture (TC16).
- Test cases: 16 now. TC15 (request not listed before approval), TC16
  (first slot clear of a turnaround is not a conflict), TC07 relabelled
  Boundary, TC02 updated for Planning.
- DOCUMENTATION.md: changelog, business rule row, fixture count.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-43_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-43_Test_Cases.xlsx
@@ -22,6 +22,8 @@
     <sheet name="TC12" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="TC13" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="TC14" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="TC15" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="TC16" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -461,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -735,7 +737,7 @@
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
@@ -968,81 +970,146 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>TC15</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>SPM-43-TC15</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>A request for an event that has not been approved yet is not shown to Venue Staff</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>AC1</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>TC16</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>SPM-43-TC16</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>A request in the first slot clear of an approved booking's turnaround is not in conflict and can be approved</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>AC3, AC7</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Boundary</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>AC</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Acceptance Criterion</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="n"/>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>Covered by</t>
-        </is>
-      </c>
-      <c r="F20" s="9" t="n"/>
-    </row>
-    <row r="21" ht="17.5" customHeight="1">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>AC1</t>
-        </is>
-      </c>
-      <c r="B21" s="11" t="inlineStr">
-        <is>
-          <t>Venue Staff can view pending booking requests.</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="9" t="n"/>
-      <c r="E21" s="11" t="inlineStr">
-        <is>
-          <t>SPM-43-TC01</t>
-        </is>
-      </c>
-      <c r="F21" s="9" t="n"/>
-    </row>
-    <row r="22" ht="31" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>AC2</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>The request displays the requested venue, date, time and event information.</t>
         </is>
       </c>
       <c r="C22" s="8" t="n"/>
       <c r="D22" s="9" t="n"/>
-      <c r="E22" s="11" t="inlineStr">
-        <is>
-          <t>SPM-43-TC01
-SPM-43-TC02</t>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Covered by</t>
         </is>
       </c>
       <c r="F22" s="9" t="n"/>
     </row>
-    <row r="23" ht="112" customHeight="1">
+    <row r="23" ht="31" customHeight="1">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>AC3</t>
+          <t>AC1</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>Venue Staff can approve the request.</t>
+          <t>Venue Staff can view pending booking requests.</t>
         </is>
       </c>
       <c r="C23" s="8" t="n"/>
       <c r="D23" s="9" t="n"/>
       <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>SPM-43-TC01
+SPM-43-TC15</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="n"/>
+    </row>
+    <row r="24" ht="31" customHeight="1">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>AC2</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>The request displays the requested venue, date, time and event information.</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="9" t="n"/>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>SPM-43-TC01
+SPM-43-TC02</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="n"/>
+    </row>
+    <row r="25" ht="125.5" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>AC3</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Venue Staff can approve the request.</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="9" t="n"/>
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>SPM-43-TC03
 SPM-43-TC04
@@ -1051,104 +1118,106 @@
 SPM-43-TC11
 SPM-43-TC12
 SPM-43-TC13
-SPM-43-TC14</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="n"/>
-    </row>
-    <row r="24" ht="44.5" customHeight="1">
-      <c r="A24" s="11" t="inlineStr">
+SPM-43-TC14
+SPM-43-TC16</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="n"/>
+    </row>
+    <row r="26" ht="44.5" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>AC4</t>
         </is>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>Venue Staff can reject the request.</t>
         </is>
       </c>
-      <c r="C24" s="8" t="n"/>
-      <c r="D24" s="9" t="n"/>
-      <c r="E24" s="11" t="inlineStr">
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>SPM-43-TC08
 SPM-43-TC11
 SPM-43-TC12</t>
         </is>
       </c>
-      <c r="F24" s="9" t="n"/>
-    </row>
-    <row r="25" ht="31" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="F26" s="9" t="n"/>
+    </row>
+    <row r="27" ht="31" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>AC5</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>Venue Staff can provide a reason when rejecting a request.</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="11" t="inlineStr">
-        <is>
-          <t>SPM-43-TC07
-SPM-43-TC08</t>
-        </is>
-      </c>
-      <c r="F25" s="9" t="n"/>
-    </row>
-    <row r="26" ht="31" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
-        <is>
-          <t>AC6</t>
-        </is>
-      </c>
-      <c r="B26" s="11" t="inlineStr">
-        <is>
-          <t>Venue Staff can suggest an alternative venue or arrangement when rejecting a request, for the Coordinator to review and act on.</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="n"/>
-      <c r="D26" s="9" t="n"/>
-      <c r="E26" s="11" t="inlineStr">
-        <is>
-          <t>SPM-43-TC09
-SPM-43-TC10</t>
-        </is>
-      </c>
-      <c r="F26" s="9" t="n"/>
-    </row>
-    <row r="27" ht="44.5" customHeight="1">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>AC7</t>
-        </is>
-      </c>
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>An approved booking request becomes a Confirmed booking — the same status referenced by Detect Venue Booking Conflicts and View Venue Availability.</t>
         </is>
       </c>
       <c r="C27" s="8" t="n"/>
       <c r="D27" s="9" t="n"/>
       <c r="E27" s="11" t="inlineStr">
         <is>
+          <t>SPM-43-TC07
+SPM-43-TC08</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="n"/>
+    </row>
+    <row r="28" ht="31" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>AC6</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Venue Staff can suggest an alternative venue or arrangement when rejecting a request, for the Coordinator to review and act on.</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="9" t="n"/>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>SPM-43-TC09
+SPM-43-TC10</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="n"/>
+    </row>
+    <row r="29" ht="58" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>AC7</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>An approved booking request becomes a Confirmed booking — the same status referenced by Detect Venue Booking Conflicts and View Venue Availability.</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="9" t="n"/>
+      <c r="E29" s="11" t="inlineStr">
+        <is>
           <t>SPM-43-TC03
 SPM-43-TC04
-SPM-43-TC05</t>
-        </is>
-      </c>
-      <c r="F27" s="9" t="n"/>
-    </row>
-    <row r="29" ht="301" customHeight="1">
-      <c r="A29" s="7" t="inlineStr">
+SPM-43-TC05
+SPM-43-TC16</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="n"/>
+    </row>
+    <row r="31" ht="301" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>Code reviewed</t>
         </is>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>src/app/bookings/page.tsx
 src/app/api/venue-bookings/route.ts
@@ -1174,16 +1243,15 @@
 prisma/seed.ts</t>
         </is>
       </c>
-      <c r="C29" s="8" t="n"/>
-      <c r="D29" s="8" t="n"/>
-      <c r="E29" s="8" t="n"/>
-      <c r="F29" s="9" t="n"/>
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="8" t="n"/>
+      <c r="E31" s="8" t="n"/>
+      <c r="F31" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="E29:F29"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="E24:F24"/>
     <mergeCell ref="B22:D22"/>
@@ -1193,12 +1261,13 @@
     <mergeCell ref="E23:F23"/>
     <mergeCell ref="E27:F27"/>
     <mergeCell ref="E22:F22"/>
-    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="E28:F28"/>
     <mergeCell ref="B1:F1"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B29:D29"/>
     <mergeCell ref="E26:F26"/>
     <mergeCell ref="B25:D25"/>
     <mergeCell ref="B24:D24"/>
-    <mergeCell ref="B20:D20"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
@@ -1215,6 +1284,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2432,13 +2503,345 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-43-TC15</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="166" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Logged in as Venue Staff Marcus Wong (marcus.wong@connectsphere.com / password123).
+Seed: 'SPM43 Policy Briefing' (status Under review, 09:00-12:00 on 18 May 2027) has a Pending request for Orchard Studio (ORC-STU) on 18 May 2027, AM. The app no longer lets a Coordinator make a request before the event is approved (SPM-54), so this one is created by the fixture script and stands for a request made before that rule.
+If it is missing, or no longer Pending because an earlier run was not reset, run: npm run fixtures:spm43 (adds or resets the SPM43 test data without a reseed).
+This case changes no data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="98.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>1. Log in as marcus.wong@connectsphere.com / password123
+2. Click 'Booking Requests' in the sidebar
+3. Look through the whole list for a card for 'SPM43 Policy Briefing'
+4. Look through the list for any card whose line under 'Requested by' reads 'Event is Submitted' or 'Event is Under review'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Request: SPM43 Policy Briefing at Orchard Studio (ORC-STU), 18 May 2027, AM
+Event status: Under review</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="71.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Step 3: There is no card for 'SPM43 Policy Briefing', although its request is Pending - a request waits for its event to be approved before Venue Staff see it.
+Step 4: There is no such card: every request listed belongs to an event that is past approval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="17.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>kayalvizhi24</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>46297</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-43-TC16</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="193" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Logged in as Venue Staff Marcus Wong (marcus.wong@connectsphere.com / password123).
+Seed: 'SPM43 Board Strategy Day' has an Approved booking at Marina Auditorium (MAR-AUD, setup 60 min, teardown 30 min) on 7 May 2027, AM + PM, so its turnaround takes 7 May Night. 'SPM43 Alumni Lecture' (status Planning, 14:00-17:00 on 8 May 2027) has a Pending request for Marina Auditorium on 8 May 2027, PM only; its own setup takes 8 May AM, the slot straight after that turnaround.
+If it is missing, or no longer Pending because an earlier run was not reset, run: npm run fixtures:spm43 (adds or resets the SPM43 test data without a reseed).
+This case changes no data: the approval is cancelled in step 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="98.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>1. Log in as marcus.wong@connectsphere.com / password123
+2. Click 'Booking Requests' in the sidebar
+3. Find the 'SPM43 Alumni Lecture' card and check its Requested slot, the Setup and Turnaround lines under it, and its badge
+4. Click 'Approve' on the 'SPM43 Alumni Lecture' card
+5. In the dialog, click 'Cancel'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Pending: SPM43 Alumni Lecture, Marina Auditorium, 8 May 2027, PM (setup: 8 May AM)
+Approved: SPM43 Board Strategy Day, Marina Auditorium, 7 May 2027, AM + PM (turnaround: 7 May Night)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="125.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Step 3: Requested reads '8 May 2027 · PM (13:00–18:00)', with 'Setup: 8 May 2027 AM (07:00–12:00)' and 'Turnaround: 8 May 2027 Night (19:00–24:00)' under it. The badge reads 'Pending', not 'Conflict', and the card has no red message.
+Step 4: The 'Approve this booking?' dialog opens, naming Marina Auditorium (MAR-AUD) and '8 May 2027 · PM (13:00–18:00)' - the request can be approved.
+Step 5: The dialog closes. The card is still in the list with the badge 'Pending' and nothing has been booked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="17.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>kayalvizhi24</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>46297</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2469,76 +2872,21 @@
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>RESOLVED 2026-10-02 (Kayal): the booking's badge reads 'Approved', as in the BPMN (docs/ConnectSphere_BPMN.drawio, gateway 'Booking approved?' -&gt; 'approved'). AC7's 'Confirmed booking' is that approved booking: the stored status is 'approved', which the availability calendar (SPM-46) shows as 'Booked' and conflict detection (SPM-44) blocks on (TC03, TC04). 'Confirmed' stays an event status only ('Confirm event' is the Coordinator's later step in both diagrams), so a booking is never labelled 'Confirmed'.</t>
+          <t>Reverting: a case that approves or rejects says so in its Preconditions ('This case changes data: run npm run fixtures:spm43 once when you finish testing …'). That command is the only reset needed and is never a reseed - it resets only the 'SPM43 …' events in place (their booking requests and decisions are dropped and recreated; each event keeps its EVT- reference), makes 'SPM43 Retire Test Room' active again and resets 'SPM43 Maintenance Room' to its one maintenance period. Nothing outside the SPM43 test data is changed by any case.</t>
         </is>
       </c>
       <c r="C2" s="11" t="n"/>
     </row>
-    <row r="3" ht="71.5" customHeight="1">
+    <row r="3" ht="85" customHeight="1">
       <c r="A3" s="11" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>RESOLVED 2026-09-18 (Kristen, Jira comment on SPM-43): notifying the Coordinator of the outcome is out of scope - notifications belong to SPM-53. No test case covers a notification, and the decision route writes none (removed 2026-10-02). The Coordinator finds the decision, reason and suggestion on the event's Venue tab (TC03, TC08, TC09, TC10).</t>
+          <t>Fixtures: scripts/seed-spm43.ts creates fourteen 'SPM43 …' events in May 2027, on base-seed venues plus the two test venues SPM43-MNT and SPM43-RET; prisma/seed.ts creates the same rows. Each event keeps its EVT- reference between runs on one database, but the number differs from one database to another, so the cases name events by title and never ask the tester to type an event address.</t>
         </is>
       </c>
       <c r="C3" s="11" t="n"/>
-    </row>
-    <row r="4" ht="58" customHeight="1">
-      <c r="A4" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="11" t="inlineStr">
-        <is>
-          <t>RESOLVED 2026-10-02 (Kayal): the suggestion is an optional venue picker plus an optional free-text 'Alternative arrangement'. It is a suggestion only - nothing is booked or requested (customer #45, #110); the Coordinator submits a new request, which SPM-42 already tests.</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="n"/>
-    </row>
-    <row r="5" ht="44.5" customHeight="1">
-      <c r="A5" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>RESOLVED 2026-10-02: a refusal whose request has left the list (SPM-43-TC12, decided in another tab) is shown at the top of the Booking Requests page instead of on the card.</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="n"/>
-    </row>
-    <row r="6" ht="98.5" customHeight="1">
-      <c r="A6" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>RESOLVED 2026-10-02 (Kayal): approval blocked by an unavailable venue and by a retired venue are tested by hand (TC13, TC14), each on its own test venue so no other tester's data is touched. Venue Staff can retire and restore a venue in the app, so TC14 does both itself. Recording an unavailability period has no screen yet (Block venue, S-23 - DOCUMENTATION.md Known Gaps), so TC13's period is created by the fixture script.</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="n"/>
-    </row>
-    <row r="7" ht="112" customHeight="1">
-      <c r="A7" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>Reverting: a case that approves or rejects says so in its Preconditions ('This case changes data: run npm run fixtures:spm43 once when you finish testing …'). That command is the only reset needed and is never a reseed - it resets only the 'SPM43 …' events in place (their booking requests and decisions are dropped and recreated; each event keeps its EVT- reference), makes 'SPM43 Retire Test Room' active again and resets 'SPM43 Maintenance Room' to its one maintenance period. Nothing outside the SPM43 test data is changed by any case.</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="n"/>
-    </row>
-    <row r="8" ht="85" customHeight="1">
-      <c r="A8" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>Fixtures: scripts/seed-spm43.ts creates twelve 'SPM43 …' events in May 2027, on base-seed venues plus the two test venues SPM43-MNT and SPM43-RET; prisma/seed.ts creates the same rows. Each event keeps its EVT- reference between runs on one database, but the number differs from one database to another, so the cases name events by title and never ask the tester to type an event address.</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2752,7 +3100,7 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Logged in as Venue Staff Marcus Wong (marcus.wong@connectsphere.com / password123).
-Seed: 'SPM43 Two-Day Forum' (status Approved, 60 people, Theatre, 11 May 2027 09:00 to 12 May 2027 17:00) has a session 'Day 2' (30 people, Classroom, 14:00-17:00 on 12 May 2027) with a Pending request for Jurong Training Room (JUR-TRN, setup 45 min, teardown 30 min).
+Seed: 'SPM43 Two-Day Forum' (status Planning, 60 people, Theatre, 11 May 2027 09:00 to 12 May 2027 17:00) has a session 'Day 2' (30 people, Classroom, 14:00-17:00 on 12 May 2027) with a Pending request for Jurong Training Room (JUR-TRN, setup 45 min, teardown 30 min).
 If it is missing, or no longer Pending because an earlier run was not reset, run: npm run fixtures:spm43 (adds or resets the SPM43 test data without a reseed).</t>
         </is>
       </c>
@@ -2792,7 +3140,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 3: The card shows 'Session: Day 2'. Requested is '12 May 2027 · PM (13:00–18:00)' with 'Setup: 12 May 2027 AM (07:00–12:00)' and 'Turnaround: 12 May 2027 Night (19:00–24:00)'. The time is labelled 'Session time' and reads '12 May 2027, 14:00–17:00' (not the event's two days). Layout is 'Classroom' and Expected attendance is '30' (the session's, not the event's Theatre and 60). Venue requirements is 'Tables in rows, power at every seat.' and 'Event is Approved' is shown under Requested by.</t>
+          <t>Step 3: The card shows 'Session: Day 2'. Requested is '12 May 2027 · PM (13:00–18:00)' with 'Setup: 12 May 2027 AM (07:00–12:00)' and 'Turnaround: 12 May 2027 Night (19:00–24:00)'. The time is labelled 'Session time' and reads '12 May 2027, 14:00–17:00' (not the event's two days). Layout is 'Classroom' and Expected attendance is '30' (the session's, not the event's Theatre and 60). Venue requirements is 'Tables in rows, power at every seat.' and 'Event is Planning' is shown under Requested by.</t>
         </is>
       </c>
     </row>

</xml_diff>